<commit_message>
Switch database from Supabase to Neon Postgres
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PM_Developer_Assignment_Components_Map.xlsx
+++ b/PM_Developer_Assignment_Components_Map.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Components Map" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="APIs Needed" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Components Map" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="APIs Needed" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -727,7 +727,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Trigger → Input → Context → Processing → AI → Output (all AI tasks on Gemini Flash, config + history in Supabase, hosted on Vercel)</t>
+          <t>Trigger → Input → Context → Processing → AI → Output (all AI tasks on Gemini Flash, config + history in Neon Postgres, hosted on Vercel)</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Edits categories, keywords, min-mentions threshold, Dev.to tags and recipient email in Supabase (no code change). New keywords get a created_at date so categories can be tagged 'recently added'.</t>
+          <t>Edits categories, keywords, min-mentions threshold, Dev.to tags and recipient email in Neon Postgres (no code change). New keywords get a created_at date so categories can be tagged 'recently added'.</t>
         </is>
       </c>
       <c r="D5" s="7" t="n"/>
@@ -818,7 +818,7 @@
     <row r="7" ht="166.5" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
         <is>
-          <t>Supabase
+          <t>Neon Postgres
 (Config + History)</t>
         </is>
       </c>
@@ -921,12 +921,13 @@
       <c r="F11" s="23" t="n"/>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>Email sent through Resend to the recipient stored in Supabase, with an idempotency key (week_key, or run id for manual runs) so retries never send duplicates (up to 3 retries with backoff). The email status is saved on the brief; the catch-up run retries email-only failures.
+          <t>Email sent through Resend to the recipient stored in Neon Postgres, with an idempotency key (week_key, or run id for manual runs) so retries never send duplicates (up to 3 retries with backoff). The email status is saved on the brief; the catch-up run retries email-only failures.
 Public dashboard on Vercel: top pain points with this/last week and trend, keyword watchlist, brief, potentially unresolved list with source links, source health, run history, Run now button.
 If every source fails, a short status email is sent instead of a brief and the run is marked failed.</t>
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="24" t="inlineStr">
         <is>
@@ -964,10 +965,11 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="62" customHeight="1">
       <c r="A15" s="31" t="inlineStr">
         <is>
-          <t>Flow in one line: Cron (Fri 08:00 IST) or Run now -&gt; function reads config from Supabase -&gt; ONE 14-day fetch from HN, Dev.to and Stack Exchange, split into current and previous 7-day windows -&gt; code verifies keyword matches, dedupes (source + post_id), counts mentions, compares weeks and labels trends -&gt; Gemini Flash classifies posts and writes the brief as JSON with post ids only -&gt; code validates it and adds all numbers and links -&gt; brief saved to Supabase, shown on the dashboard and emailed to Sumit. Counting is done in code, never by the AI.</t>
+          <t>Flow in one line: Cron (Fri 08:00 IST) or Run now -&gt; function reads config from Neon Postgres -&gt; ONE 14-day fetch from HN, Dev.to and Stack Exchange, split into current and previous 7-day windows -&gt; code verifies keyword matches, dedupes (source + post_id), counts mentions, compares weeks and labels trends -&gt; Gemini Flash classifies posts and writes the brief as JSON with post ids only -&gt; code validates it and adds all numbers and links -&gt; brief saved to Neon Postgres, shown on the dashboard and emailed to Sumit. Counting is done in code, never by the AI.</t>
         </is>
       </c>
     </row>
@@ -1030,22 +1032,22 @@
       </c>
       <c r="B2" s="33" t="inlineStr">
         <is>
-          <t>Supabase (REST / JS client)</t>
+          <t>Neon Postgres (serverless driver)</t>
         </is>
       </c>
       <c r="C2" s="33" t="inlineStr">
         <is>
-          <t>Config (topics, settings) and history (posts, weekly_stats, briefs, job_runs)</t>
+          <t>Config (topics, settings) and history (posts, weekly_stats, briefs, runs)</t>
         </is>
       </c>
       <c r="D2" s="33" t="inlineStr">
         <is>
-          <t>Yes: project URL + service key</t>
+          <t>Yes: DATABASE_URL (Neon connection string)</t>
         </is>
       </c>
       <c r="E2" s="33" t="inlineStr">
         <is>
-          <t>supabase.from('topics').select('*').eq('active', true)</t>
+          <t>sql`select * from topics where active`  (@neondatabase/serverless, DATABASE_URL)</t>
         </is>
       </c>
     </row>
@@ -1085,7 +1087,7 @@
       </c>
       <c r="C4" s="33" t="inlineStr">
         <is>
-          <t>No keyword search: fetch by tag (tags kept in Supabase), filter keywords and dates in code</t>
+          <t>No keyword search: fetch by tag (tags kept in Neon Postgres), filter keywords and dates in code</t>
         </is>
       </c>
       <c r="D4" s="33" t="inlineStr">

</xml_diff>

<commit_message>
Deploy to Vercel, sync Excel, add SUBMISSION.md
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PM_Developer_Assignment_Components_Map.xlsx
+++ b/PM_Developer_Assignment_Components_Map.xlsx
@@ -879,7 +879,7 @@
 3. Upsert posts and post_matches. Mention = one unique source + post_id per category per window by created_at, so a post matching several keywords in one category counts once. Same rule at keyword level.
 4. Percent change in code, only when previous &gt; 0. Trend label order: failed request -&gt; 'Incomplete, no trend'; 0 and 0 -&gt; 'No mentions (confirmed zero)'; total below min_mentions -&gt; 'Insufficient data'; previous 0 -&gt; 'New'; now 0 -&gt; 'Dropped to zero'; else Up / Down / Flat.
 5. Categories with topics added in the last 14 days are tagged 'recently added' (their baseline is real because both windows are always fetched).
-6. 'Potentially unresolved' evidence by source: Stack Overflow no answers / no accepted answer; HN question or complaint with 0-1 comments; Dev.to only help/discuss posts with 0 comments. Never 'unsolved'.
+6. 'Potentially unresolved' evidence by source: Stack Overflow no answers, or no accepted or upvoted answer (Stack Exchange is_answered = false); HN question or complaint with 0-1 comments; Dev.to only help/discuss posts with 0 comments. Never 'unsolved'.
 7. Validate Gemini JSON; renderer adds every number, trend and link from the database; failures logged to runs and shown as a dashboard banner.</t>
         </is>
       </c>
@@ -927,7 +927,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="24" t="inlineStr">
         <is>
@@ -965,7 +964,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="62" customHeight="1">
       <c r="A15" s="31" t="inlineStr">
         <is>
@@ -1097,7 +1095,7 @@
       </c>
       <c r="E4" s="33" t="inlineStr">
         <is>
-          <t>https://dev.to/api/articles?tag=codereview&amp;per_page=30</t>
+          <t>https://dev.to/api/articles?tag=codereview&amp;per_page=100&amp;page=1  (paged up to 5 pages per tag, stopping when a page is older than the window)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Final polish: unresolved rules, thin evidence, consistent history, run notes, Neon wording, Excel sync
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PM_Developer_Assignment_Components_Map.xlsx
+++ b/PM_Developer_Assignment_Components_Map.xlsx
@@ -778,7 +778,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Optional: presses Run now on the dashboard (passcode + 5-minute cooldown) -&gt; /api/run-now, anchor = now</t>
+          <t>Optional: presses Run now on the dashboard (passcode + 5-minute cooldown) -&gt; POST /api/run-now (anchor = now); while it runs the panel polls GET /api/run-status every 2 s and shows the live stage (fetch, count, analyse, write, email)</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -828,9 +828,10 @@
         <is>
           <t>topics: category, keyword, active, created_at
 settings: min_mentions, flat threshold, Dev.to tags, classify cap, recipient email
-posts: unique on source + post_id, with cached AI labels (relevant, sentiment, pain_point, seeking_help)
+posts: unique on source + post_id, with cached AI labels (saved once, never repeated) (relevant, sentiment, pain_point, seeking_help)
 post_matches: source + post_id + category + keyword
-weekly_stats, briefs, runs (week_key, status, attempts, source_status, error)</t>
+weekly_stats, briefs, runs (week_key, status, attempts, stage, source_status, error)
+Config and history live in Neon Postgres, the Supabase/Neon option allowed by the course stack.</t>
         </is>
       </c>
       <c r="E7" s="12" t="n"/>
@@ -878,8 +879,8 @@
 2. Verify matches in code: the keyword must really appear in the title or snippet (word-boundary match, e.g. 'CI/CD'); the APIs are fuzzy.
 3. Upsert posts and post_matches. Mention = one unique source + post_id per category per window by created_at, so a post matching several keywords in one category counts once. Same rule at keyword level.
 4. Percent change in code, only when previous &gt; 0. Trend label order: failed request -&gt; 'Incomplete, no trend'; 0 and 0 -&gt; 'No mentions (confirmed zero)'; total below min_mentions -&gt; 'Insufficient data'; previous 0 -&gt; 'New'; now 0 -&gt; 'Dropped to zero'; else Up / Down / Flat.
-5. Categories with topics added in the last 14 days are tagged 'recently added' (their baseline is real because both windows are always fetched).
-6. 'Potentially unresolved' evidence by source: Stack Overflow no answers, or no accepted or upvoted answer (Stack Exchange is_answered = false); HN question or complaint with 0-1 comments; Dev.to only help/discuss posts with 0 comments. Never 'unsolved'.
+5. Categories with topics added in the last 14 days are tagged 'recently added' (their baseline is real because both windows are always fetched). A category backed by only 1 or 2 posts is labelled 'thin evidence'.
+6. 'Potentially unresolved' evidence by source: Stack Overflow no answers, or no accepted or upvoted answer (Stack Exchange is_answered = false); HN question or complaint with 0-1 comments; Dev.to only help/discuss posts with 0 comments. Show HN, blog and announcement posts are excluded and every candidate needs a question or complaint signal. Never 'unsolved'.
 7. Validate Gemini JSON; renderer adds every number, trend and link from the database; failures logged to runs and shown as a dashboard banner.</t>
         </is>
       </c>
@@ -922,7 +923,7 @@
       <c r="G11" s="8" t="inlineStr">
         <is>
           <t>Email sent through Resend to the recipient stored in Neon Postgres, with an idempotency key (week_key, or run id for manual runs) so retries never send duplicates (up to 3 retries with backoff). The email status is saved on the brief; the catch-up run retries email-only failures.
-Public dashboard on Vercel: top pain points with this/last week and trend, keyword watchlist, brief, potentially unresolved list with source links, source health, run history, Run now button.
+Public dashboard on Vercel: top pain points with this/last week and trend, keyword watchlist, brief, potentially unresolved list with source links, source health, run history (with a plain-words note for each partial run), Run now button with live stage progress.
 If every source fails, a short status email is sent instead of a brief and the run is marked failed.</t>
         </is>
       </c>
@@ -1035,7 +1036,7 @@
       </c>
       <c r="C2" s="33" t="inlineStr">
         <is>
-          <t>Config (topics, settings) and history (posts, weekly_stats, briefs, runs)</t>
+          <t>Config (topics, settings) and history (posts, weekly_stats, briefs, runs incl. stage). Neon Postgres is the Supabase/Neon option allowed by the course stack</t>
         </is>
       </c>
       <c r="D2" s="33" t="inlineStr">
@@ -1185,7 +1186,7 @@
       </c>
       <c r="C8" s="33" t="inlineStr">
         <is>
-          <t>Primary Friday 08:00 IST run, catch-up run, run-now route and the public dashboard URL (production deployment only)</t>
+          <t>Primary Friday 08:00 IST run (/api/cron/weekly), catch-up run (/api/cron/weekly?catchup=1), POST /api/run-now, GET /api/run-status and the public dashboard URL (production deployment only)</t>
         </is>
       </c>
       <c r="D8" s="33" t="inlineStr">
@@ -1210,7 +1211,7 @@
       </c>
       <c r="C9" s="33" t="inlineStr">
         <is>
-          <t>Public repo for submission; auto-deploys to Vercel</t>
+          <t>Public repo for submission; deployed to Vercel production with the Vercel CLI</t>
         </is>
       </c>
       <c r="D9" s="33" t="inlineStr">

</xml_diff>

<commit_message>
Topics page docs, Excel, end-to-end test script
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PM_Developer_Assignment_Components_Map.xlsx
+++ b/PM_Developer_Assignment_Components_Map.xlsx
@@ -783,7 +783,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Edits categories, keywords, min-mentions threshold, Dev.to tags and recipient email in Neon Postgres (no code change). New keywords get a created_at date so categories can be tagged 'recently added'.</t>
+          <t>Manages categories and keywords on the /topics page (behind the Run now passcode, stored in Neon Postgres): add, rename, move, switch on/off, never delete. A new or re-typed keyword is backfilled for 14 days straight away (3 sources, no Gemini), so its trend shows right away. Other settings (min-mentions threshold, Dev.to tags, recipient email) are rows in Neon. New keywords get a created_at date so categories can be tagged 'recently added'.</t>
         </is>
       </c>
       <c r="D5" s="7" t="n"/>
@@ -826,11 +826,11 @@
       <c r="C7" s="12" t="n"/>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>topics: category, keyword, active, created_at
+          <t>categories: id, name, active | topics: id, category_id, keyword, active, created_at (permanent ids; posts, weekly stats and history point to the ids, so renames keep history)
 settings: min_mentions, flat threshold, Dev.to tags, classify cap, recipient email
 posts: unique on source + post_id, with cached AI labels (saved once, never repeated) (relevant, sentiment, pain_point, seeking_help)
-post_matches: source + post_id + category + keyword
-weekly_stats, briefs, runs (week_key, status, attempts, stage, source_status, error)
+post_matches: source + post_id + topic_id
+weekly_stats, briefs, runs (week_key, status, attempts, stage, source_status, error; run_type scheduled / manual / backfill)
 Config and history live in Neon Postgres, the Supabase/Neon option allowed by the course stack.</t>
         </is>
       </c>
@@ -1036,7 +1036,7 @@
       </c>
       <c r="C2" s="33" t="inlineStr">
         <is>
-          <t>Config (topics, settings) and history (posts, weekly_stats, briefs, runs incl. stage). Neon Postgres is the Supabase/Neon option allowed by the course stack</t>
+          <t>Config (categories, topics with permanent ids, settings) and history (posts, weekly_stats, briefs, runs incl. stage). Neon Postgres is the Supabase/Neon option allowed by the course stack</t>
         </is>
       </c>
       <c r="D2" s="33" t="inlineStr">

</xml_diff>